<commit_message>
Actualizacion automatica de datos - lun 25/05/2026 14:53:06,39
</commit_message>
<xml_diff>
--- a/Cronograma de Tareas/Cronograma Mayo.xlsx
+++ b/Cronograma de Tareas/Cronograma Mayo.xlsx
@@ -2871,18 +2871,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="K31:L31"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="K31:L31"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B7">
     <cfRule type="duplicateValues" dxfId="136" priority="30"/>
@@ -3792,18 +3792,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="K32:L32"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="K32:L32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B7">
     <cfRule type="duplicateValues" dxfId="101" priority="30"/>
@@ -4719,18 +4719,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="K32:L32"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="K32:L32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B7">
     <cfRule type="duplicateValues" dxfId="66" priority="30"/>
@@ -5606,18 +5606,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="K30:L30"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="duplicateValues" dxfId="31" priority="32"/>

</xml_diff>